<commit_message>
feat: implementar hoja Reporte Auxiliar IVA con aviso legal y corrección de bases en exportación Excel
</commit_message>
<xml_diff>
--- a/templates/dian-excel-template.xlsx
+++ b/templates/dian-excel-template.xlsx
@@ -6,14 +6,15 @@
   <sheets>
     <sheet sheetId="1" name="Facturas DIAN" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Detallado" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Datos de terceros" state="visible" r:id="rId6"/>
+    <sheet sheetId="3" name="Reporte Auxiliar IVA" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Datos de terceros" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="81">
   <si>
     <t>ContaGO - Exportador DIAN</t>
   </si>
@@ -163,6 +164,48 @@
   </si>
   <si>
     <t>Precio unitario (incluye impuestos)</t>
+  </si>
+  <si>
+    <t>ContaGO - Reporte Auxiliar IVA</t>
+  </si>
+  <si>
+    <t>AVISO LEGAL: Esta herramienta proporciona un reporte auxiliar basado en los datos extraídos. ContaGO NO liquida impuestos. Es responsabilidad exclusiva del usuario revisar y validar esta información antes de cualquier presentación ante autoridades tributarias.</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>Tipo documento</t>
+  </si>
+  <si>
+    <t>Número factura</t>
+  </si>
+  <si>
+    <t>Razón Social Emisor</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Bases de IVAS al 19%</t>
+  </si>
+  <si>
+    <t>IVAS del 19%</t>
+  </si>
+  <si>
+    <t>Bases IVAS 5%</t>
+  </si>
+  <si>
+    <t>IVAS 5%</t>
+  </si>
+  <si>
+    <t>Bases sin IVA</t>
+  </si>
+  <si>
+    <t>IVA 0%</t>
+  </si>
+  <si>
+    <t>Factura Electrónica de Venta</t>
   </si>
   <si>
     <t>ContaGO - Datos de terceros</t>
@@ -220,7 +263,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -237,6 +280,11 @@
       <b/>
       <color rgb="FF000000"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FFFF0000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -264,13 +312,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -992,6 +1043,141 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
+    <tabColor rgb="FF92D050"/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="15"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="12" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="4" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+    </row>
+    <row r="5" ht="25" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6">
+        <v>1000000</v>
+      </c>
+      <c r="H6">
+        <v>190000</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A4:L4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
     <tabColor rgb="FFF59E0B"/>
   </sheetPr>
   <dimension ref="A1:M3"/>
@@ -1011,7 +1197,7 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1034,31 +1220,31 @@
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>6</v>
@@ -1075,7 +1261,7 @@
         <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="D3" t="s">
         <v>27</v>
@@ -1084,22 +1270,22 @@
         <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>61</v>
+        <v>75</v>
       </c>
       <c r="G3" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="H3" t="s">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="I3" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="J3" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="K3" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="L3" t="s">
         <v>29</v>

</xml_diff>